<commit_message>
Home: tolto "CABRU —" dal titolo della pagina e dal title SEO (IT+EN)
Recepite le due correzioni scritte da Carlo nell'XLS del 29.08:
- SEO Title: "CABRU — Offre prodotti..." -> "CABRU Offre prodotti..."
- Titolo pagina (H1): via il prefisso "CABRU — "
Applicate anche a og:title e alla home EN, per tenere le due lingue allineate.
XLS rigenerato dopo la modifica; backup della versione con le correzioni.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_tooling/CABRU_testi_IT_da_correggere.xlsx
+++ b/_tooling/CABRU_testi_IT_da_correggere.xlsx
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>CABRU — Offre prodotti per laboratori di ricerca in ambito scientifico</t>
+          <t>CABRU Offre prodotti per laboratori di ricerca in ambito scientifico</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr"/>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr"/>
     </row>
-    <row r="8" ht="51" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Titolo pagina</t>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>CABRU — Reagenti e prodotti per laboratori di ricerca nell'ambito delle scienze della vita e per laboratori di controllo qualità di industrie biotecnologiche, farmaceutiche, alimentari, cosmetiche</t>
+          <t>Reagenti e prodotti per laboratori di ricerca nell'ambito delle scienze della vita e per laboratori di controllo qualità di industrie biotecnologiche, farmaceutiche, alimentari, cosmetiche</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Home: "CABRU —" tolto anche dall'occhiello e dalle descrizioni (IT+EN)
Completa la correzione di stamattina, che aveva toccato solo il title SEO e
l'H1: l'occhiello riprende la forma del title (senza trattino), la meta
description quella dell'H1 (senza il prefisso), e con lei og:description e le
due descrizioni nei dati strutturati, che portavano lo stesso testo.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_tooling/CABRU_testi_IT_da_correggere.xlsx
+++ b/_tooling/CABRU_testi_IT_da_correggere.xlsx
@@ -4478,7 +4478,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr"/>
     </row>
-    <row r="5" ht="51" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>SEO — Meta description</t>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>CABRU — Reagenti e prodotti per laboratori di ricerca nell'ambito delle scienze della vita e per laboratori di controllo qualità di industrie biotecnologiche, farmaceutiche, alimentari, cosmetiche</t>
+          <t>Reagenti e prodotti per laboratori di ricerca nell'ambito delle scienze della vita e per laboratori di controllo qualità di industrie biotecnologiche, farmaceutiche, alimentari, cosmetiche</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr"/>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>CABRU — Offre prodotti per laboratori di ricerca in ambito scientifico</t>
+          <t>CABRU Offre prodotti per laboratori di ricerca in ambito scientifico</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Home: logo grande in apertura, banda di invito al contatto, pallino lingua tondo
Il logo apre la home in grande e al primo scorrimento si scambia con
quello dell'intestazione: due dissolvenze della stessa durata avviate
insieme, non una riduzione in movimento. Il file grande e' tagliato dal
sorgente ad alta risoluzione e ha il fondo trasparente, perche' sul
grigio dell'apertura il bianco si vedrebbe come un rettangolo.

Nuova banda prima dei contatti: dice cosa si guadagna a farsi
consigliare e offre le tre strade separate — telefono, scheda di
contatto e mail dal proprio programma di posta. Finora il pulsante
"Invia una email" apriva comunque la scheda: la terza strada non
esisteva.

L'informativa privacy diceva che solo l'email era obbligatoria: da oggi
lo sono anche nome e cognome, in italiano e in inglese.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_tooling/CABRU_testi_IT_da_correggere.xlsx
+++ b/_tooling/CABRU_testi_IT_da_correggere.xlsx
@@ -4426,7 +4426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5138,25 +5138,25 @@
     <row r="56" ht="21" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Occhiello</t>
+          <t>Testo</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Dove trovarci</t>
+          <t>Un confronto prima dell'ordine evita la referenza sbagliata.</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr"/>
     </row>
-    <row r="57" ht="21" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
-        <is>
-          <t>Titolo sezione</t>
-        </is>
-      </c>
-      <c r="B57" s="11" t="inlineStr">
-        <is>
-          <t>Contatti</t>
+    <row r="57" ht="51" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Testo</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Dicci l'applicazione, la matrice e il formato che ti servono: individuiamo la referenza adatta fra i produttori che rappresentiamo, verifichiamo disponibilità e tempi di consegna, e seguiamo la richiesta fino alla consegna con un unico referente.</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr"/>
@@ -5164,25 +5164,25 @@
     <row r="58" ht="21" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Contatto</t>
+          <t>Occhiello</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Via Enrico Forlanini 52 20862 Arcore (MB)</t>
+          <t>Dove trovarci</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr"/>
     </row>
     <row r="59" ht="21" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>Contatto</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>039 6013988</t>
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Titolo sezione</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>Contatti</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr"/>
@@ -5195,33 +5195,33 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
+          <t>Via Enrico Forlanini 52 20862 Arcore (MB)</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr"/>
+    </row>
+    <row r="61" ht="21" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Contatto</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>039 6013988</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr"/>
+    </row>
+    <row r="62" ht="21" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Contatto</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
           <t>info@cabru.it</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr"/>
-    </row>
-    <row r="61" ht="21" customHeight="1">
-      <c r="A61" s="10" t="inlineStr">
-        <is>
-          <t>Sottotitolo</t>
-        </is>
-      </c>
-      <c r="B61" s="11" t="inlineStr">
-        <is>
-          <t>Richieste di informazioni</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr"/>
-    </row>
-    <row r="62" ht="36" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>Testo</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>Per un preventivo, verificare la disponibilità di un prodotto o per un'informazione tecnica, CABRU è sempre a disposizione e risponde nel più breve tempo possibile.</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr"/>
@@ -5229,12 +5229,12 @@
     <row r="63" ht="21" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Titolo sezione</t>
+          <t>Sottotitolo</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Qualità certificata, dal produttore al laboratorio</t>
+          <t>Richieste di informazioni</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr"/>
@@ -5247,10 +5247,36 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
+          <t>Per un preventivo, verificare la disponibilità di un prodotto o per un'informazione tecnica, CABRU è sempre a disposizione e risponde nel più breve tempo possibile.</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr"/>
+    </row>
+    <row r="65" ht="21" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Titolo sezione</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>Qualità certificata, dal produttore al laboratorio</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr"/>
+    </row>
+    <row r="66" ht="36" customHeight="1">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>Testo</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
           <t>CABRU opera con un sistema di gestione della qualità certificato ISO 9001 e rappresenta produttori con sistemi qualità certificati (ISO 9001 e/o ISO 13485).</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr"/>
+      <c r="C66" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>